<commit_message>
Rephrase quasi-LBO section into original voice; update Summary sheet narrative to match
</commit_message>
<xml_diff>
--- a/financial-models/FOUR_Financial_Model.xlsx
+++ b/financial-models/FOUR_Financial_Model.xlsx
@@ -26,12 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="297">
   <si>
     <t xml:space="preserve">SHIFT4 PAYMENTS (FOUR) — Investment Model</t>
   </si>
   <si>
-    <t xml:space="preserve">Institutional-Grade Financial Analysis | Quasi-LBO Framework</t>
+    <t xml:space="preserve">Nicholas Steiglehner | University of Michigan, Ross School of Business | Quasi-LBO Framework</t>
   </si>
   <si>
     <t xml:space="preserve">COMPANY OVERVIEW</t>
@@ -161,6 +161,21 @@
   </si>
   <si>
     <t xml:space="preserve">Bull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALYTICAL FRAMEWORK — QUASI-LBO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Private equity returns follow a predictable decomposition: the business grows revenue, expands margins, and is eventually sold at some multiple of earnings. Along the way, free cash flow retires debt. The equity check compounds from two directions simultaneously — the business itself getting bigger, and the debt layer staying roughly fixed while enterprise value climbs above it. Every incremental dollar of EV creation flows disproportionately to equity holders. That mechanic doesn't disappear in public markets. It just gets ignored.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The cleaner starting point is enterprise value, not earnings per share. Build a forward EBITDA projection. Apply a conservative exit multiple. Then work backward to equity value, netting out net debt after accounting for FCF accumulation and share count reduction over the holding period. P/E ratios are a snapshot of today's interest burden — they don't capture the quiet migration of value from the debt tranche to the equity tranche that plays out over years as cash flows accrue. That migration isn't financial engineering. It's arithmetic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three conditions are required for the framework to work: (1) a high-quality business that reliably compounds free cash flow, (2) a manageable and declining debt stack, and (3) an EV multiple that doesn't price in the compounding. When those three conditions are satisfied, the equity payoff profile becomes structurally asymmetric — downside anchored to business quality, upside amplified by the math of value migration. FOUR satisfies all three today at $42.56.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When the five questions get five affirmative answers, you're not looking at a leveraged bet. You're looking at something that resembles a small private buyout hiding in the public market at a discount. That's not a reason to be aggressive — it's a reason to be patient. The business compounds, FCF accrues, and the value follows. The weighing machine, given enough time, tends to respect the arithmetic.</t>
   </si>
   <si>
     <t xml:space="preserve">SHEET NAVIGATION</t>
@@ -908,7 +923,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0\x"/>
@@ -916,12 +931,11 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="170" formatCode="0"/>
-    <numFmt numFmtId="171" formatCode="\$#,##0"/>
-    <numFmt numFmtId="172" formatCode="0.00\x"/>
-    <numFmt numFmtId="173" formatCode="0.0"/>
-    <numFmt numFmtId="174" formatCode="0\x"/>
+    <numFmt numFmtId="171" formatCode="0.00\x"/>
+    <numFmt numFmtId="172" formatCode="0.0"/>
+    <numFmt numFmtId="173" formatCode="0\x"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1007,6 +1021,22 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <u val="single"/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
@@ -1078,13 +1108,6 @@
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1129,7 +1152,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1139,7 +1162,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8F4F8"/>
-        <bgColor rgb="FFE8F4E8"/>
+        <bgColor rgb="FFEBF3FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -1151,13 +1174,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1B474D"/>
-        <bgColor rgb="FF444444"/>
+        <bgColor rgb="FF1A3C6B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8F4E8"/>
         <bgColor rgb="FFE8F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A3C6B"/>
+        <bgColor rgb="FF1B474D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF3FA"/>
+        <bgColor rgb="FFE8F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFC0"/>
+        <bgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
     <fill>
@@ -1246,7 +1287,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="78">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1339,15 +1380,31 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1355,7 +1412,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1363,7 +1428,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1375,11 +1440,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1395,23 +1460,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1427,46 +1492,42 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="171" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="172" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1475,7 +1536,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1483,11 +1544,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1499,11 +1560,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1515,7 +1576,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1523,19 +1584,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1568,12 +1629,12 @@
       <rgbColor rgb="FF888888"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FFA13544"/>
-      <rgbColor rgb="FFE8F4E8"/>
+      <rgbColor rgb="FFFFFFC0"/>
       <rgbColor rgb="FFE8F4F8"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF006494"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFEBF3FA"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1583,7 +1644,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFE8F4E8"/>
       <rgbColor rgb="FFD4EDDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -1598,13 +1659,13 @@
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666666"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF1B474D"/>
+      <rgbColor rgb="FF1A3C6B"/>
       <rgbColor rgb="FF437A22"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FFA84B2F"/>
       <rgbColor rgb="FF7A39BB"/>
-      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF1B474D"/>
       <rgbColor rgb="FF444444"/>
     </indexedColors>
   </colors>
@@ -1792,7 +1853,7 @@
     <tabColor rgb="FF1B474D"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:J33"/>
+  <dimension ref="B2:J42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
@@ -2075,117 +2136,186 @@
         <v>0.653175282353036</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="4" t="s">
+    <row r="20" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="23" t="s">
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+    </row>
+    <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+    </row>
+    <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="23" t="s">
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+    </row>
+    <row r="24" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="24" t="s">
-        <v>49</v>
-      </c>
+      <c r="C24" s="24"/>
       <c r="D24" s="24"/>
       <c r="E24" s="24"/>
       <c r="F24" s="24"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="23" t="s">
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+    </row>
+    <row r="25" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+    </row>
+    <row r="26" customFormat="false" ht="3.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="24" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="23" t="s">
+      <c r="C32" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="24" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="23" t="s">
+      <c r="C33" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="24" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="23" t="s">
+      <c r="C34" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C28" s="24" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="25" t="s">
+      <c r="C35" s="30" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="26" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="29" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="25" t="s">
+      <c r="C36" s="30" t="s">
         <v>60</v>
       </c>
     </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="31" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="31" t="s">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B23:J23"/>
     <mergeCell ref="C23:F23"/>
+    <mergeCell ref="B24:J24"/>
     <mergeCell ref="C24:F24"/>
+    <mergeCell ref="B25:J25"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="C26:F26"/>
     <mergeCell ref="C27:F27"/>
     <mergeCell ref="C28:F28"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B23" location="'Operating Model'!B2" display="Operating Model"/>
-    <hyperlink ref="B24" location="'Cash Waterfall'!B2" display="Quarterly Cash Waterfall"/>
-    <hyperlink ref="B25" location="'Buyback &amp; Shares'!B2" display="Buyback &amp; Share Count"/>
-    <hyperlink ref="B26" location="'Valuation'!B2" display="Valuation Scenarios"/>
-    <hyperlink ref="B27" location="'Peer Comps'!B2" display="Peer Comps"/>
-    <hyperlink ref="B28" location="'Float Analysis'!B2" display="Float Analysis"/>
-    <hyperlink ref="B32" r:id="rId1" display="Data: https://perplexity.ai/finance/FOUR"/>
+    <hyperlink ref="B23" location="'Operating Model'!B2" display="The cleaner starting point is enterprise value, not earnings per share. Build a forward EBITDA projection. Apply a conservative exit multiple. Then work backward to equity value, netting out net debt after accounting for FCF accumulation and share count reduction over the holding period. P/E ratios are a snapshot of today's interest burden — they don't capture the quiet migration of value from the debt tranche to the equity tranche that plays out over years as cash flows accrue. That migration isn't financial engineering. It's arithmetic."/>
+    <hyperlink ref="B24" location="'Cash Waterfall'!B2" display="Three conditions are required for the framework to work: (1) a high-quality business that reliably compounds free cash flow, (2) a manageable and declining debt stack, and (3) an EV multiple that doesn't price in the compounding. When those three conditions are satisfied, the equity payoff profile becomes structurally asymmetric — downside anchored to business quality, upside amplified by the math of value migration. FOUR satisfies all three today at $42.56."/>
+    <hyperlink ref="B25" location="'Buyback &amp; Shares'!B2" display="When the five questions get five affirmative answers, you're not looking at a leveraged bet. You're looking at something that resembles a small private buyout hiding in the public market at a discount. That's not a reason to be aggressive — it's a reason to be patient. The business compounds, FCF accrues, and the value follows. The weighing machine, given enough time, tends to respect the arithmetic."/>
+    <hyperlink ref="B32" r:id="rId1" display="Operating Model"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2212,22 +2342,22 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="27" t="s">
-        <v>61</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
+      <c r="B2" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2240,40 +2370,40 @@
       <c r="K3" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="28" t="s">
-        <v>63</v>
+      <c r="B5" s="34" t="s">
+        <v>68</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="29" t="s">
-        <v>73</v>
+      <c r="B6" s="35" t="s">
+        <v>78</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>1990</v>
@@ -2287,7 +2417,7 @@
       <c r="F6" s="10" t="n">
         <v>4180</v>
       </c>
-      <c r="G6" s="30" t="n">
+      <c r="G6" s="36" t="n">
         <v>5225</v>
       </c>
       <c r="H6" s="10" t="n">
@@ -2305,9 +2435,9 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="31"/>
+        <v>79</v>
+      </c>
+      <c r="C7" s="37"/>
       <c r="D7" s="15" t="n">
         <f aca="false">(D6-C6)/C6</f>
         <v>0.28643216080402</v>
@@ -2343,7 +2473,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>780</v>
@@ -2357,7 +2487,7 @@
       <c r="F8" s="10" t="n">
         <v>1976</v>
       </c>
-      <c r="G8" s="30" t="n">
+      <c r="G8" s="36" t="n">
         <v>2550</v>
       </c>
       <c r="H8" s="10" t="n">
@@ -2375,9 +2505,9 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="31"/>
+        <v>81</v>
+      </c>
+      <c r="C9" s="37"/>
       <c r="D9" s="15" t="n">
         <f aca="false">(D8-C8)/C8</f>
         <v>0.307692307692308</v>
@@ -2413,7 +2543,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>470</v>
@@ -2445,7 +2575,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C12" s="15" t="n">
         <f aca="false">C11/C6</f>
@@ -2485,8 +2615,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="29" t="s">
-        <v>79</v>
+      <c r="B14" s="35" t="s">
+        <v>84</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>269</v>
@@ -2500,10 +2630,10 @@
       <c r="F14" s="10" t="n">
         <v>817</v>
       </c>
-      <c r="G14" s="30" t="n">
+      <c r="G14" s="36" t="n">
         <v>1307</v>
       </c>
-      <c r="H14" s="30" t="n">
+      <c r="H14" s="36" t="n">
         <v>1580</v>
       </c>
       <c r="J14" s="10" t="n">
@@ -2518,9 +2648,9 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" s="31"/>
+        <v>85</v>
+      </c>
+      <c r="C15" s="37"/>
       <c r="D15" s="15" t="n">
         <f aca="false">IF(C14=0,"-",(D14-C14)/C14)</f>
         <v>0.360594795539033</v>
@@ -2556,7 +2686,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C16" s="15" t="n">
         <f aca="false">C14/C6</f>
@@ -2596,33 +2726,33 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="G17" s="33" t="n">
+      <c r="B17" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" s="39" t="n">
         <v>1190</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="29" t="s">
-        <v>83</v>
-      </c>
-      <c r="C19" s="34" t="n">
+      <c r="B19" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="40" t="n">
         <v>-105</v>
       </c>
-      <c r="D19" s="34" t="n">
+      <c r="D19" s="40" t="n">
         <v>251</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="40" t="n">
         <v>311</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="40" t="n">
         <v>499</v>
       </c>
-      <c r="G19" s="30" t="n">
+      <c r="G19" s="36" t="n">
         <v>585</v>
       </c>
-      <c r="H19" s="30" t="n">
+      <c r="H19" s="36" t="n">
         <v>750</v>
       </c>
       <c r="I19" s="10" t="n">
@@ -2637,7 +2767,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C20" s="15" t="n">
         <f aca="false">IF(C6=0,"-",C19/C6)</f>
@@ -2678,7 +2808,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>72</v>
@@ -2692,7 +2822,7 @@
       <c r="F22" s="10" t="n">
         <v>209</v>
       </c>
-      <c r="G22" s="30" t="n">
+      <c r="G22" s="36" t="n">
         <v>250</v>
       </c>
       <c r="H22" s="10" t="n">
@@ -2710,9 +2840,9 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="31"/>
+        <v>91</v>
+      </c>
+      <c r="C23" s="37"/>
       <c r="D23" s="15" t="n">
         <f aca="false">(D22-C22)/C22</f>
         <v>0.513888888888889</v>
@@ -2748,81 +2878,81 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C24" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="C24" s="41" t="n">
         <v>61</v>
       </c>
-      <c r="D24" s="35" t="n">
+      <c r="D24" s="41" t="n">
         <v>62</v>
       </c>
-      <c r="E24" s="35" t="n">
+      <c r="E24" s="41" t="n">
         <v>61</v>
       </c>
-      <c r="F24" s="35" t="n">
+      <c r="F24" s="41" t="n">
         <v>60</v>
       </c>
-      <c r="G24" s="35" t="n">
+      <c r="G24" s="41" t="n">
         <v>61</v>
       </c>
-      <c r="H24" s="35" t="n">
+      <c r="H24" s="41" t="n">
         <v>61</v>
       </c>
-      <c r="I24" s="35" t="n">
+      <c r="I24" s="41" t="n">
         <v>61</v>
       </c>
-      <c r="J24" s="35" t="n">
+      <c r="J24" s="41" t="n">
         <v>61</v>
       </c>
-      <c r="K24" s="35" t="n">
+      <c r="K24" s="41" t="n">
         <v>61</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="36"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="36"/>
-      <c r="J25" s="36"/>
-      <c r="K25" s="36"/>
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="25" t="s">
-        <v>58</v>
+      <c r="B27" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="26" t="s">
-        <v>59</v>
+      <c r="B28" s="32" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="25" t="s">
-        <v>60</v>
+      <c r="B29" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="37" t="s">
-        <v>88</v>
+      <c r="B31" s="43" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="38" t="s">
-        <v>89</v>
+      <c r="B32" s="44" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="39" t="s">
-        <v>90</v>
+      <c r="B33" s="45" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="40" t="s">
-        <v>91</v>
+      <c r="B34" s="46" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2858,24 +2988,24 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="27" t="s">
-        <v>92</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
+      <c r="B2" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2892,259 +3022,259 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="9"/>
       <c r="C5" s="9" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10" t="n">
         <v>964</v>
       </c>
-      <c r="E6" s="41" t="n">
+      <c r="E6" s="47" t="n">
         <f aca="false">D13</f>
         <v>556</v>
       </c>
-      <c r="F6" s="41" t="n">
+      <c r="F6" s="47" t="n">
         <f aca="false">E13</f>
         <v>414</v>
       </c>
-      <c r="G6" s="41" t="n">
+      <c r="G6" s="47" t="n">
         <f aca="false">F13</f>
         <v>561</v>
       </c>
-      <c r="H6" s="41" t="n">
+      <c r="H6" s="47" t="n">
         <f aca="false">G13</f>
         <v>631</v>
       </c>
-      <c r="I6" s="41" t="n">
+      <c r="I6" s="47" t="n">
         <f aca="false">H13</f>
         <v>746</v>
       </c>
-      <c r="J6" s="41" t="n">
+      <c r="J6" s="47" t="n">
         <f aca="false">I13</f>
         <v>936</v>
       </c>
-      <c r="K6" s="41" t="n">
+      <c r="K6" s="47" t="n">
         <f aca="false">J13</f>
         <v>573</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C7" s="12"/>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="36" t="n">
         <v>70</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="36" t="n">
         <v>148</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="36" t="n">
         <v>222</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="36" t="n">
         <v>145</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="36" t="n">
         <v>115</v>
       </c>
-      <c r="I7" s="30" t="n">
+      <c r="I7" s="36" t="n">
         <v>190</v>
       </c>
-      <c r="J7" s="30" t="n">
+      <c r="J7" s="36" t="n">
         <v>270</v>
       </c>
-      <c r="K7" s="30" t="n">
+      <c r="K7" s="36" t="n">
         <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C8" s="34" t="n">
+        <v>110</v>
+      </c>
+      <c r="C8" s="40" t="n">
         <v>-305</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="40" t="n">
         <v>-255</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="40" t="n">
         <v>-440</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="42"/>
-      <c r="D9" s="34" t="n">
+        <v>111</v>
+      </c>
+      <c r="C9" s="48"/>
+      <c r="D9" s="40" t="n">
         <v>-223</v>
       </c>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="42"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="48"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" s="42"/>
-      <c r="D10" s="42"/>
-      <c r="E10" s="34" t="n">
+        <v>112</v>
+      </c>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="40" t="n">
         <v>150</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="40" t="n">
         <v>-75</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="40" t="n">
         <v>-75</v>
       </c>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="42"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="34" t="n">
+        <v>113</v>
+      </c>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="40" t="n">
         <v>-633</v>
       </c>
-      <c r="K11" s="42"/>
+      <c r="K11" s="48"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="43"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="49"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="29" t="s">
-        <v>109</v>
+      <c r="B13" s="35" t="s">
+        <v>114</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>964</v>
       </c>
-      <c r="D13" s="44" t="n">
+      <c r="D13" s="50" t="n">
         <f aca="false">SUM(D6:D11)</f>
         <v>556</v>
       </c>
-      <c r="E13" s="44" t="n">
+      <c r="E13" s="50" t="n">
         <f aca="false">SUM(E6:E11)</f>
         <v>414</v>
       </c>
-      <c r="F13" s="44" t="n">
+      <c r="F13" s="50" t="n">
         <f aca="false">SUM(F6:F11)</f>
         <v>561</v>
       </c>
-      <c r="G13" s="44" t="n">
+      <c r="G13" s="50" t="n">
         <f aca="false">SUM(G6:G11)</f>
         <v>631</v>
       </c>
-      <c r="H13" s="44" t="n">
+      <c r="H13" s="50" t="n">
         <f aca="false">SUM(H6:H11)</f>
         <v>746</v>
       </c>
-      <c r="I13" s="44" t="n">
+      <c r="I13" s="50" t="n">
         <f aca="false">SUM(I6:I11)</f>
         <v>936</v>
       </c>
-      <c r="J13" s="44" t="n">
+      <c r="J13" s="50" t="n">
         <f aca="false">SUM(J6:J11)</f>
         <v>573</v>
       </c>
-      <c r="K13" s="44" t="n">
+      <c r="K13" s="50" t="n">
         <f aca="false">SUM(K6:K11)</f>
         <v>748</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C15" s="30" t="n">
+        <v>115</v>
+      </c>
+      <c r="C15" s="36" t="n">
         <v>304</v>
       </c>
-      <c r="D15" s="30" t="n">
+      <c r="D15" s="36" t="n">
         <v>233</v>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="36" t="n">
         <v>330</v>
       </c>
-      <c r="F15" s="30" t="n">
+      <c r="F15" s="36" t="n">
         <v>409</v>
       </c>
-      <c r="G15" s="30" t="n">
+      <c r="G15" s="36" t="n">
         <v>335</v>
       </c>
-      <c r="H15" s="30" t="n">
+      <c r="H15" s="36" t="n">
         <v>290</v>
       </c>
-      <c r="I15" s="30" t="n">
+      <c r="I15" s="36" t="n">
         <v>395</v>
       </c>
-      <c r="J15" s="30" t="n">
+      <c r="J15" s="36" t="n">
         <v>490</v>
       </c>
-      <c r="K15" s="30" t="n">
+      <c r="K15" s="36" t="n">
         <v>405</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>970</v>
@@ -3176,121 +3306,121 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C17" s="45" t="n">
+        <v>117</v>
+      </c>
+      <c r="C17" s="10" t="n">
         <v>4543</v>
       </c>
-      <c r="D17" s="45" t="n">
+      <c r="D17" s="10" t="n">
         <v>4547</v>
       </c>
-      <c r="E17" s="45" t="n">
+      <c r="E17" s="10" t="n">
         <v>4544</v>
       </c>
-      <c r="F17" s="45" t="n">
+      <c r="F17" s="10" t="n">
         <v>4547</v>
       </c>
-      <c r="G17" s="45" t="n">
+      <c r="G17" s="10" t="n">
         <v>4539</v>
       </c>
-      <c r="H17" s="45" t="n">
+      <c r="H17" s="10" t="n">
         <v>4540</v>
       </c>
-      <c r="I17" s="45" t="n">
+      <c r="I17" s="10" t="n">
         <v>4539</v>
       </c>
-      <c r="J17" s="45" t="n">
+      <c r="J17" s="10" t="n">
         <v>3906</v>
       </c>
-      <c r="K17" s="45" t="n">
+      <c r="K17" s="10" t="n">
         <v>3906</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="46" t="n">
+      <c r="C18" s="51" t="n">
         <f aca="false">C17-C13</f>
         <v>3579</v>
       </c>
-      <c r="D18" s="46" t="n">
+      <c r="D18" s="51" t="n">
         <f aca="false">D17-D13</f>
         <v>3991</v>
       </c>
-      <c r="E18" s="46" t="n">
+      <c r="E18" s="51" t="n">
         <f aca="false">E17-E13</f>
         <v>4130</v>
       </c>
-      <c r="F18" s="46" t="n">
+      <c r="F18" s="51" t="n">
         <f aca="false">F17-F13</f>
         <v>3986</v>
       </c>
-      <c r="G18" s="46" t="n">
+      <c r="G18" s="51" t="n">
         <f aca="false">G17-G13</f>
         <v>3908</v>
       </c>
-      <c r="H18" s="46" t="n">
+      <c r="H18" s="51" t="n">
         <f aca="false">H17-H13</f>
         <v>3794</v>
       </c>
-      <c r="I18" s="46" t="n">
+      <c r="I18" s="51" t="n">
         <f aca="false">I17-I13</f>
         <v>3603</v>
       </c>
-      <c r="J18" s="46" t="n">
+      <c r="J18" s="51" t="n">
         <f aca="false">J17-J13</f>
         <v>3333</v>
       </c>
-      <c r="K18" s="46" t="n">
+      <c r="K18" s="51" t="n">
         <f aca="false">K17-K13</f>
         <v>3158</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="C19" s="47" t="n">
+      <c r="B19" s="35" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="52" t="n">
         <f aca="false">C18/C16</f>
         <v>3.68969072164948</v>
       </c>
-      <c r="D19" s="47" t="n">
+      <c r="D19" s="52" t="n">
         <f aca="false">D18/D16</f>
         <v>3.72990654205608</v>
       </c>
-      <c r="E19" s="47" t="n">
+      <c r="E19" s="52" t="n">
         <f aca="false">E18/E16</f>
         <v>3.52991452991453</v>
       </c>
-      <c r="F19" s="47" t="n">
+      <c r="F19" s="52" t="n">
         <f aca="false">F18/F16</f>
         <v>3.06144393241167</v>
       </c>
-      <c r="G19" s="47" t="n">
+      <c r="G19" s="52" t="n">
         <f aca="false">G18/G16</f>
         <v>2.99005355776588</v>
       </c>
-      <c r="H19" s="47" t="n">
+      <c r="H19" s="52" t="n">
         <f aca="false">H18/H16</f>
         <v>2.71971326164875</v>
       </c>
-      <c r="I19" s="47" t="n">
+      <c r="I19" s="52" t="n">
         <f aca="false">I18/I16</f>
         <v>2.37978863936592</v>
       </c>
-      <c r="J19" s="47" t="n">
+      <c r="J19" s="52" t="n">
         <f aca="false">J18/J16</f>
         <v>2.19565217391304</v>
       </c>
-      <c r="K19" s="47" t="n">
+      <c r="K19" s="52" t="n">
         <f aca="false">K18/K16</f>
         <v>1.99873417721519</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -3303,102 +3433,102 @@
       <c r="K21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="48"/>
-      <c r="J22" s="48"/>
-      <c r="K22" s="48"/>
+      <c r="B22" s="53" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="53"/>
+      <c r="I22" s="53"/>
+      <c r="J22" s="53"/>
+      <c r="K22" s="53"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="48"/>
-      <c r="J23" s="48"/>
-      <c r="K23" s="48"/>
+      <c r="B23" s="53" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" s="53"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
+      <c r="G23" s="53"/>
+      <c r="H23" s="53"/>
+      <c r="I23" s="53"/>
+      <c r="J23" s="53"/>
+      <c r="K23" s="53"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="48" t="s">
-        <v>117</v>
-      </c>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-      <c r="J24" s="48"/>
-      <c r="K24" s="48"/>
+      <c r="B24" s="53" t="s">
+        <v>122</v>
+      </c>
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
+      <c r="K24" s="53"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="48" t="s">
-        <v>118</v>
-      </c>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
-      <c r="I25" s="48"/>
-      <c r="J25" s="48"/>
-      <c r="K25" s="48"/>
+      <c r="B25" s="53" t="s">
+        <v>123</v>
+      </c>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
+      <c r="G25" s="53"/>
+      <c r="H25" s="53"/>
+      <c r="I25" s="53"/>
+      <c r="J25" s="53"/>
+      <c r="K25" s="53"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="48" t="s">
-        <v>119</v>
-      </c>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="48"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="48"/>
-      <c r="J26" s="48"/>
-      <c r="K26" s="48"/>
+      <c r="B26" s="53" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="53"/>
+      <c r="J26" s="53"/>
+      <c r="K26" s="53"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="48" t="s">
-        <v>120</v>
-      </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="48"/>
-      <c r="K27" s="48"/>
+      <c r="B27" s="53" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
+      <c r="G27" s="53"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="53"/>
+      <c r="J27" s="53"/>
+      <c r="K27" s="53"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="25" t="s">
-        <v>58</v>
+      <c r="B29" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="26" t="s">
-        <v>59</v>
+      <c r="B30" s="32" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="25" t="s">
-        <v>60</v>
+      <c r="B31" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -3441,18 +3571,18 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="27" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="B2" s="33" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -3462,7 +3592,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -3470,23 +3600,23 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="49" t="n">
+        <v>133</v>
+      </c>
+      <c r="C7" s="54" t="n">
         <v>4.3</v>
       </c>
       <c r="D7" s="10" t="n">
@@ -3499,9 +3629,9 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C8" s="49" t="n">
+        <v>134</v>
+      </c>
+      <c r="C8" s="54" t="n">
         <v>4.7</v>
       </c>
       <c r="D8" s="10" t="n">
@@ -3514,9 +3644,9 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C9" s="49" t="n">
+        <v>135</v>
+      </c>
+      <c r="C9" s="54" t="n">
         <v>9.8</v>
       </c>
       <c r="D9" s="10" t="n">
@@ -3529,24 +3659,24 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C10" s="50" t="n">
+        <v>136</v>
+      </c>
+      <c r="C10" s="55" t="n">
         <f aca="false">SUM(C7:C9)</f>
         <v>18.8</v>
       </c>
-      <c r="D10" s="46" t="n">
+      <c r="D10" s="51" t="n">
         <f aca="false">SUM(D7:D9)</f>
         <v>1000</v>
       </c>
-      <c r="E10" s="51" t="n">
+      <c r="E10" s="56" t="n">
         <f aca="false">D10/C10</f>
         <v>53.1914893617021</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3556,53 +3686,53 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="9"/>
       <c r="C15" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C16" s="49" t="n">
+        <v>142</v>
+      </c>
+      <c r="C16" s="54" t="n">
         <v>86.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C17" s="31"/>
-      <c r="D17" s="49" t="n">
+        <v>143</v>
+      </c>
+      <c r="C17" s="37"/>
+      <c r="D17" s="54" t="n">
         <v>-18.8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="52" t="n">
+        <v>144</v>
+      </c>
+      <c r="C18" s="37"/>
+      <c r="D18" s="57" t="n">
         <v>5.8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D19" s="50" t="n">
+        <v>145</v>
+      </c>
+      <c r="D19" s="55" t="n">
         <f aca="false">C16+D17+D18</f>
         <v>73.5</v>
       </c>
-      <c r="E19" s="53" t="n">
+      <c r="E19" s="58" t="n">
         <f aca="false">D19-C16</f>
         <v>-13</v>
       </c>
@@ -3613,39 +3743,39 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C20" s="49" t="n">
+        <v>146</v>
+      </c>
+      <c r="C20" s="54" t="n">
         <v>10</v>
       </c>
-      <c r="D20" s="49" t="n">
+      <c r="D20" s="54" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="C21" s="50" t="n">
+      <c r="B21" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" s="55" t="n">
         <f aca="false">C16+C20</f>
         <v>96.5</v>
       </c>
-      <c r="D21" s="54" t="n">
+      <c r="D21" s="59" t="n">
         <f aca="false">D19+D20</f>
         <v>83.5</v>
       </c>
-      <c r="E21" s="53" t="n">
+      <c r="E21" s="58" t="n">
         <f aca="false">D21-C21</f>
         <v>-13</v>
       </c>
-      <c r="F21" s="55" t="n">
+      <c r="F21" s="60" t="n">
         <f aca="false">E21/C21</f>
         <v>-0.134715025906736</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -3655,18 +3785,18 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="9"/>
       <c r="C25" s="9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="5" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>500</v>
@@ -3680,54 +3810,54 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C27" s="49" t="n">
+        <v>150</v>
+      </c>
+      <c r="C27" s="54" t="n">
         <v>86.5</v>
       </c>
-      <c r="D27" s="49" t="n">
+      <c r="D27" s="54" t="n">
         <v>73.5</v>
       </c>
-      <c r="E27" s="49" t="n">
+      <c r="E27" s="54" t="n">
         <v>74</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C28" s="49" t="n">
+        <v>151</v>
+      </c>
+      <c r="C28" s="54" t="n">
         <v>96.5</v>
       </c>
-      <c r="D28" s="49" t="n">
+      <c r="D28" s="54" t="n">
         <v>83.5</v>
       </c>
-      <c r="E28" s="49" t="n">
+      <c r="E28" s="54" t="n">
         <v>84</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="29" t="s">
-        <v>147</v>
-      </c>
-      <c r="C29" s="56" t="n">
+      <c r="B29" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="61" t="n">
         <f aca="false">C26/C27</f>
         <v>5.78034682080925</v>
       </c>
-      <c r="D29" s="56" t="n">
+      <c r="D29" s="61" t="n">
         <f aca="false">D26/D27</f>
         <v>7.95918367346939</v>
       </c>
-      <c r="E29" s="56" t="n">
+      <c r="E29" s="61" t="n">
         <f aca="false">E26/E27</f>
         <v>10.1351351351351</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C30" s="31"/>
+        <v>153</v>
+      </c>
+      <c r="C30" s="37"/>
       <c r="D30" s="15" t="n">
         <f aca="false">(D29-C29)/C29</f>
         <v>0.376938775510204</v>
@@ -3738,27 +3868,27 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="57" t="s">
-        <v>149</v>
-      </c>
-      <c r="C32" s="57"/>
-      <c r="D32" s="57"/>
-      <c r="E32" s="57"/>
-      <c r="F32" s="57"/>
+      <c r="B32" s="62" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="25" t="s">
-        <v>58</v>
+      <c r="B34" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="26" t="s">
-        <v>59</v>
+      <c r="B35" s="32" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="25" t="s">
-        <v>60</v>
+      <c r="B36" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -3798,20 +3928,20 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
+      <c r="B2" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -3823,7 +3953,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -3855,7 +3985,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>23</v>
@@ -3863,7 +3993,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="5" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>7</v>
@@ -3879,15 +4009,15 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="5" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -3896,44 +4026,44 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C16" s="58" t="n">
+        <v>168</v>
+      </c>
+      <c r="C16" s="63" t="n">
         <v>10.14</v>
       </c>
-      <c r="D16" s="51" t="n">
+      <c r="D16" s="56" t="n">
         <f aca="false">C16*15</f>
         <v>152.1</v>
       </c>
-      <c r="E16" s="51" t="n">
+      <c r="E16" s="56" t="n">
         <f aca="false">C16*18</f>
         <v>182.52</v>
       </c>
-      <c r="F16" s="51" t="n">
+      <c r="F16" s="56" t="n">
         <f aca="false">C16*20</f>
         <v>202.8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D17" s="15" t="n">
         <f aca="false">(D16-42.56)/42.56</f>
@@ -3950,7 +4080,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -3961,45 +4091,45 @@
       <c r="I20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="59" t="s">
-        <v>166</v>
-      </c>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="59"/>
-      <c r="H21" s="59"/>
-      <c r="I21" s="59"/>
+      <c r="B21" s="64" t="s">
+        <v>171</v>
+      </c>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
+      <c r="E21" s="64"/>
+      <c r="F21" s="64"/>
+      <c r="G21" s="64"/>
+      <c r="H21" s="64"/>
+      <c r="I21" s="64"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="C22" s="60" t="n">
+        <v>172</v>
+      </c>
+      <c r="C22" s="65" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="60" t="n">
+      <c r="D22" s="65" t="n">
         <v>9</v>
       </c>
-      <c r="E22" s="60" t="n">
+      <c r="E22" s="65" t="n">
         <v>10</v>
       </c>
-      <c r="F22" s="60" t="n">
+      <c r="F22" s="65" t="n">
         <v>11</v>
       </c>
-      <c r="G22" s="60" t="n">
+      <c r="G22" s="65" t="n">
         <v>12</v>
       </c>
-      <c r="H22" s="60" t="n">
+      <c r="H22" s="65" t="n">
         <v>13</v>
       </c>
-      <c r="I22" s="60" t="n">
+      <c r="I22" s="65" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="61" t="n">
+      <c r="B23" s="66" t="n">
         <v>0.08</v>
       </c>
       <c r="C23" s="13" t="n">
@@ -4032,7 +4162,7 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="61" t="n">
+      <c r="B24" s="66" t="n">
         <v>0.1</v>
       </c>
       <c r="C24" s="13" t="n">
@@ -4065,7 +4195,7 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="61" t="n">
+      <c r="B25" s="66" t="n">
         <v>0.12</v>
       </c>
       <c r="C25" s="13" t="n">
@@ -4076,7 +4206,7 @@
         <f aca="false">(1307*(1+$B25)^4*D$22-2000)/63</f>
         <v>262.052511613968</v>
       </c>
-      <c r="E25" s="62" t="n">
+      <c r="E25" s="67" t="n">
         <f aca="false">(1307*(1+$B25)^4*E$22-2000)/63</f>
         <v>294.696794209524</v>
       </c>
@@ -4098,7 +4228,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="61" t="n">
+      <c r="B26" s="66" t="n">
         <v>0.15</v>
       </c>
       <c r="C26" s="13" t="n">
@@ -4131,7 +4261,7 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="61" t="n">
+      <c r="B27" s="66" t="n">
         <v>0.18</v>
       </c>
       <c r="C27" s="13" t="n">
@@ -4164,7 +4294,7 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="61" t="n">
+      <c r="B28" s="66" t="n">
         <v>0.21</v>
       </c>
       <c r="C28" s="13" t="n">
@@ -4197,20 +4327,20 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="59" t="s">
-        <v>168</v>
-      </c>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="59"/>
-      <c r="H30" s="59"/>
-      <c r="I30" s="59"/>
+      <c r="B30" s="64" t="s">
+        <v>173</v>
+      </c>
+      <c r="C30" s="64"/>
+      <c r="D30" s="64"/>
+      <c r="E30" s="64"/>
+      <c r="F30" s="64"/>
+      <c r="G30" s="64"/>
+      <c r="H30" s="64"/>
+      <c r="I30" s="64"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -4219,18 +4349,18 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="5" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="5" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4238,7 +4368,7 @@
         <v>35</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4246,62 +4376,62 @@
         <v>34</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="5" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="5" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="5" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="25" t="s">
-        <v>58</v>
+      <c r="B44" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="26" t="s">
-        <v>59</v>
+      <c r="B45" s="32" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="25" t="s">
-        <v>60</v>
+      <c r="B46" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -4362,22 +4492,22 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
+      <c r="B2" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -4397,257 +4527,257 @@
         <v>8</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>10</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="63" t="s">
-        <v>195</v>
-      </c>
-      <c r="C6" s="63" t="s">
-        <v>196</v>
-      </c>
-      <c r="D6" s="64" t="s">
+      <c r="B6" s="68" t="s">
+        <v>200</v>
+      </c>
+      <c r="C6" s="68" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="64" t="s">
+      <c r="E6" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="64" t="s">
-        <v>197</v>
-      </c>
-      <c r="G6" s="64" t="s">
-        <v>198</v>
-      </c>
-      <c r="H6" s="64" t="s">
-        <v>199</v>
-      </c>
-      <c r="I6" s="64" t="s">
-        <v>200</v>
-      </c>
-      <c r="J6" s="64" t="s">
-        <v>201</v>
-      </c>
-      <c r="K6" s="64" t="s">
+      <c r="F6" s="69" t="s">
         <v>202</v>
       </c>
+      <c r="G6" s="69" t="s">
+        <v>203</v>
+      </c>
+      <c r="H6" s="69" t="s">
+        <v>204</v>
+      </c>
+      <c r="I6" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="J6" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="K6" s="69" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="65" t="s">
-        <v>203</v>
-      </c>
-      <c r="C7" s="65" t="s">
-        <v>204</v>
-      </c>
-      <c r="D7" s="66" t="s">
-        <v>205</v>
-      </c>
-      <c r="E7" s="66" t="s">
-        <v>206</v>
-      </c>
-      <c r="F7" s="66" t="s">
-        <v>207</v>
-      </c>
-      <c r="G7" s="66" t="s">
+      <c r="B7" s="70" t="s">
         <v>208</v>
       </c>
-      <c r="H7" s="66" t="s">
+      <c r="C7" s="70" t="s">
         <v>209</v>
       </c>
-      <c r="I7" s="66" t="s">
+      <c r="D7" s="71" t="s">
         <v>210</v>
       </c>
-      <c r="J7" s="66" t="s">
+      <c r="E7" s="71" t="s">
         <v>211</v>
       </c>
-      <c r="K7" s="66" t="s">
+      <c r="F7" s="71" t="s">
         <v>212</v>
       </c>
+      <c r="G7" s="71" t="s">
+        <v>213</v>
+      </c>
+      <c r="H7" s="71" t="s">
+        <v>214</v>
+      </c>
+      <c r="I7" s="71" t="s">
+        <v>215</v>
+      </c>
+      <c r="J7" s="71" t="s">
+        <v>216</v>
+      </c>
+      <c r="K7" s="71" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="65" t="s">
-        <v>213</v>
-      </c>
-      <c r="C8" s="65" t="s">
-        <v>214</v>
-      </c>
-      <c r="D8" s="66" t="s">
-        <v>215</v>
-      </c>
-      <c r="E8" s="66" t="s">
-        <v>216</v>
-      </c>
-      <c r="F8" s="66" t="s">
-        <v>217</v>
-      </c>
-      <c r="G8" s="66" t="s">
+      <c r="B8" s="70" t="s">
         <v>218</v>
       </c>
-      <c r="H8" s="66" t="s">
+      <c r="C8" s="70" t="s">
         <v>219</v>
       </c>
-      <c r="I8" s="66" t="s">
+      <c r="D8" s="71" t="s">
         <v>220</v>
       </c>
-      <c r="J8" s="66" t="s">
+      <c r="E8" s="71" t="s">
         <v>221</v>
       </c>
-      <c r="K8" s="66" t="s">
+      <c r="F8" s="71" t="s">
         <v>222</v>
       </c>
+      <c r="G8" s="71" t="s">
+        <v>223</v>
+      </c>
+      <c r="H8" s="71" t="s">
+        <v>224</v>
+      </c>
+      <c r="I8" s="71" t="s">
+        <v>225</v>
+      </c>
+      <c r="J8" s="71" t="s">
+        <v>226</v>
+      </c>
+      <c r="K8" s="71" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="65" t="s">
-        <v>223</v>
-      </c>
-      <c r="C9" s="65" t="s">
-        <v>224</v>
-      </c>
-      <c r="D9" s="66" t="s">
-        <v>225</v>
-      </c>
-      <c r="E9" s="66" t="s">
-        <v>226</v>
-      </c>
-      <c r="F9" s="66" t="s">
-        <v>227</v>
-      </c>
-      <c r="G9" s="66" t="s">
+      <c r="B9" s="70" t="s">
         <v>228</v>
       </c>
-      <c r="H9" s="66" t="s">
+      <c r="C9" s="70" t="s">
         <v>229</v>
       </c>
-      <c r="I9" s="66" t="s">
+      <c r="D9" s="71" t="s">
         <v>230</v>
       </c>
-      <c r="J9" s="66" t="s">
+      <c r="E9" s="71" t="s">
         <v>231</v>
       </c>
-      <c r="K9" s="66" t="s">
+      <c r="F9" s="71" t="s">
         <v>232</v>
       </c>
+      <c r="G9" s="71" t="s">
+        <v>233</v>
+      </c>
+      <c r="H9" s="71" t="s">
+        <v>234</v>
+      </c>
+      <c r="I9" s="71" t="s">
+        <v>235</v>
+      </c>
+      <c r="J9" s="71" t="s">
+        <v>236</v>
+      </c>
+      <c r="K9" s="71" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="65" t="s">
-        <v>233</v>
-      </c>
-      <c r="C10" s="65" t="s">
-        <v>234</v>
-      </c>
-      <c r="D10" s="66" t="s">
-        <v>235</v>
-      </c>
-      <c r="E10" s="66" t="s">
-        <v>236</v>
-      </c>
-      <c r="F10" s="66" t="s">
-        <v>237</v>
-      </c>
-      <c r="G10" s="66" t="s">
+      <c r="B10" s="70" t="s">
         <v>238</v>
       </c>
-      <c r="H10" s="66" t="s">
+      <c r="C10" s="70" t="s">
         <v>239</v>
       </c>
-      <c r="I10" s="66" t="s">
+      <c r="D10" s="71" t="s">
         <v>240</v>
       </c>
-      <c r="J10" s="66" t="s">
+      <c r="E10" s="71" t="s">
         <v>241</v>
       </c>
-      <c r="K10" s="66" t="s">
+      <c r="F10" s="71" t="s">
         <v>242</v>
       </c>
+      <c r="G10" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="H10" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="I10" s="71" t="s">
+        <v>245</v>
+      </c>
+      <c r="J10" s="71" t="s">
+        <v>246</v>
+      </c>
+      <c r="K10" s="71" t="s">
+        <v>247</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="65" t="s">
-        <v>243</v>
-      </c>
-      <c r="C11" s="65" t="s">
-        <v>244</v>
-      </c>
-      <c r="D11" s="66" t="s">
-        <v>245</v>
-      </c>
-      <c r="E11" s="66" t="s">
-        <v>246</v>
-      </c>
-      <c r="F11" s="66" t="s">
-        <v>247</v>
-      </c>
-      <c r="G11" s="66" t="s">
+      <c r="B11" s="70" t="s">
         <v>248</v>
       </c>
-      <c r="H11" s="66" t="s">
+      <c r="C11" s="70" t="s">
         <v>249</v>
       </c>
-      <c r="I11" s="66" t="s">
+      <c r="D11" s="71" t="s">
         <v>250</v>
       </c>
-      <c r="J11" s="66" t="s">
+      <c r="E11" s="71" t="s">
         <v>251</v>
       </c>
-      <c r="K11" s="66" t="s">
+      <c r="F11" s="71" t="s">
         <v>252</v>
       </c>
+      <c r="G11" s="71" t="s">
+        <v>253</v>
+      </c>
+      <c r="H11" s="71" t="s">
+        <v>254</v>
+      </c>
+      <c r="I11" s="71" t="s">
+        <v>255</v>
+      </c>
+      <c r="J11" s="71" t="s">
+        <v>256</v>
+      </c>
+      <c r="K11" s="71" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="65" t="s">
-        <v>253</v>
-      </c>
-      <c r="C12" s="65" t="s">
-        <v>254</v>
-      </c>
-      <c r="D12" s="66" t="s">
-        <v>255</v>
-      </c>
-      <c r="E12" s="66" t="s">
-        <v>256</v>
-      </c>
-      <c r="F12" s="66" t="s">
-        <v>257</v>
-      </c>
-      <c r="G12" s="66" t="s">
+      <c r="B12" s="70" t="s">
         <v>258</v>
       </c>
-      <c r="H12" s="66" t="s">
-        <v>258</v>
-      </c>
-      <c r="I12" s="66" t="s">
-        <v>258</v>
-      </c>
-      <c r="J12" s="66" t="s">
-        <v>258</v>
-      </c>
-      <c r="K12" s="66" t="s">
-        <v>258</v>
+      <c r="C12" s="70" t="s">
+        <v>259</v>
+      </c>
+      <c r="D12" s="71" t="s">
+        <v>260</v>
+      </c>
+      <c r="E12" s="71" t="s">
+        <v>261</v>
+      </c>
+      <c r="F12" s="71" t="s">
+        <v>262</v>
+      </c>
+      <c r="G12" s="71" t="s">
+        <v>263</v>
+      </c>
+      <c r="H12" s="71" t="s">
+        <v>263</v>
+      </c>
+      <c r="I12" s="71" t="s">
+        <v>263</v>
+      </c>
+      <c r="J12" s="71" t="s">
+        <v>263</v>
+      </c>
+      <c r="K12" s="71" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -4660,22 +4790,22 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="67" t="s">
-        <v>260</v>
-      </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
-      <c r="I15" s="67"/>
-      <c r="J15" s="67"/>
-      <c r="K15" s="67"/>
+      <c r="B15" s="72" t="s">
+        <v>265</v>
+      </c>
+      <c r="C15" s="72"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="72"/>
+      <c r="G15" s="72"/>
+      <c r="H15" s="72"/>
+      <c r="I15" s="72"/>
+      <c r="J15" s="72"/>
+      <c r="K15" s="72"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="4" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -4689,26 +4819,26 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="68" t="s">
+      <c r="G18" s="73" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="5" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
-      <c r="G19" s="68" t="s">
-        <v>264</v>
+      <c r="G19" s="73" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4719,7 +4849,7 @@
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
-      <c r="G20" s="68" t="s">
+      <c r="G20" s="73" t="s">
         <v>15</v>
       </c>
     </row>
@@ -4731,23 +4861,23 @@
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
-      <c r="G21" s="68" t="s">
+      <c r="G21" s="73" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="25" t="s">
-        <v>58</v>
+      <c r="B24" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="26" t="s">
-        <v>59</v>
+      <c r="B25" s="32" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="25" t="s">
-        <v>60</v>
+      <c r="B26" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -4790,17 +4920,17 @@
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="27" t="s">
-        <v>265</v>
-      </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
+      <c r="B2" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -4809,7 +4939,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -4817,216 +4947,216 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9"/>
       <c r="C6" s="9" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="65" t="s">
-        <v>269</v>
-      </c>
-      <c r="C7" s="49" t="n">
+      <c r="B7" s="70" t="s">
+        <v>274</v>
+      </c>
+      <c r="C7" s="54" t="n">
         <v>84.6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="65" t="s">
-        <v>270</v>
-      </c>
-      <c r="C8" s="49" t="n">
+      <c r="B8" s="70" t="s">
+        <v>275</v>
+      </c>
+      <c r="C8" s="54" t="n">
         <v>-3.4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="65"/>
-      <c r="C9" s="49" t="n">
+      <c r="B9" s="70"/>
+      <c r="C9" s="54" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="C11" s="54" t="n">
+        <v>276</v>
+      </c>
+      <c r="C11" s="59" t="n">
         <f aca="false">SUM(C7:C9)</f>
         <v>81.2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="4" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>273</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="C15" s="49" t="n">
+        <v>279</v>
+      </c>
+      <c r="C15" s="54" t="n">
         <v>23.5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="C16" s="49" t="n">
+        <v>280</v>
+      </c>
+      <c r="C16" s="54" t="n">
         <v>6.8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="C17" s="49" t="n">
+        <v>281</v>
+      </c>
+      <c r="C17" s="54" t="n">
         <v>6.6</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="C18" s="49" t="n">
+        <v>282</v>
+      </c>
+      <c r="C18" s="54" t="n">
         <v>5.6</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C19" s="49" t="n">
+        <v>283</v>
+      </c>
+      <c r="C19" s="54" t="n">
         <v>2.6</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="C20" s="54" t="n">
+        <v>284</v>
+      </c>
+      <c r="C20" s="59" t="n">
         <f aca="false">SUM(C15:C19)</f>
         <v>45.1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="59" t="s">
-        <v>280</v>
-      </c>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
+      <c r="B21" s="64" t="s">
+        <v>285</v>
+      </c>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="4" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="C24" s="69" t="n">
+        <v>287</v>
+      </c>
+      <c r="C24" s="74" t="n">
         <f aca="false">C11</f>
         <v>81.2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="C25" s="69" t="n">
+        <v>288</v>
+      </c>
+      <c r="C25" s="74" t="n">
         <f aca="false">-C20</f>
         <v>-45.1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="29" t="s">
-        <v>284</v>
-      </c>
-      <c r="C26" s="54" t="n">
+      <c r="B26" s="35" t="s">
+        <v>289</v>
+      </c>
+      <c r="C26" s="59" t="n">
         <f aca="false">C24+C25</f>
         <v>36.1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="C28" s="49" t="n">
+        <v>290</v>
+      </c>
+      <c r="C28" s="54" t="n">
         <v>16.2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="29" t="s">
-        <v>286</v>
-      </c>
-      <c r="C29" s="70" t="n">
+      <c r="B29" s="35" t="s">
+        <v>291</v>
+      </c>
+      <c r="C29" s="75" t="n">
         <f aca="false">C28/C26</f>
         <v>0.448753462603878</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="4" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="C32" s="52" t="n">
+        <v>293</v>
+      </c>
+      <c r="C32" s="57" t="n">
         <v>10.5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="C33" s="50" t="n">
+        <v>294</v>
+      </c>
+      <c r="C33" s="55" t="n">
         <f aca="false">C26-C32</f>
         <v>25.6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="29" t="s">
-        <v>290</v>
-      </c>
-      <c r="C34" s="71" t="n">
+      <c r="B34" s="35" t="s">
+        <v>295</v>
+      </c>
+      <c r="C34" s="76" t="n">
         <f aca="false">C28/C33</f>
         <v>0.6328125</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="72" t="s">
-        <v>291</v>
-      </c>
-      <c r="C36" s="72"/>
-      <c r="D36" s="72"/>
-      <c r="E36" s="72"/>
+      <c r="B36" s="77" t="s">
+        <v>296</v>
+      </c>
+      <c r="C36" s="77"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="25" t="s">
-        <v>58</v>
+      <c r="B38" s="31" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="26" t="s">
-        <v>59</v>
+      <c r="B39" s="32" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="25" t="s">
-        <v>60</v>
+      <c r="B40" s="31" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>